<commit_message>
Atualização base de indicadores
</commit_message>
<xml_diff>
--- a/Bases/base_indicadores_rj.xlsx
+++ b/Bases/base_indicadores_rj.xlsx
@@ -23,31 +23,31 @@
     <t xml:space="preserve">densidade_demografica</t>
   </si>
   <si>
-    <t xml:space="preserve">urbanizacao</t>
+    <t xml:space="preserve">IU</t>
   </si>
   <si>
     <t xml:space="preserve">razao_dependencia</t>
   </si>
   <si>
-    <t xml:space="preserve">proporcao_idosos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">raca_predominante</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prop_chefes_mulheres</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prop_mulher</t>
+    <t xml:space="preserve">IPI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IPR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IPCM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IRMH</t>
   </si>
   <si>
     <t xml:space="preserve">tamanho_medio_dom</t>
   </si>
   <si>
-    <t xml:space="preserve">coleta_lixo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">prop_esgoto_adequado</t>
+    <t xml:space="preserve">ICLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IEA</t>
   </si>
   <si>
     <t xml:space="preserve">IRRSM</t>

</xml_diff>